<commit_message>
Incorporate user-confirmed HPA data for CALML5 tissue expression
The user checked proteinatlas.org herself (blocked in this sandbox)
and shared screenshots showing CALML5 is genuinely and substantially
expressed in vagina (protein Low, RNA 272.7 nTPM via GTEx) and cervix
(protein Medium, RNA 198.9 nTPM), specifically in squamous epithelial
cells (not glandular) - matching the cornification hypothesis already
established.

Document what this does and doesn't resolve: it confirms CALML5 is a
real, robustly-expressed gene in the relevant human tissue type (not
a technical artifact of gene annotation), which makes the near-zero/
non-zero split seen in the rat SUI Untreated/Treated samples more
plausibly a real biological induction pattern - but it's baseline
GTEx tissue data, not a POP/SUI-vs-control comparison, so it doesn't
directly validate the differential expression finding, and the n=3
per group statistical power limitation in the rat DESeq2 comparison
is unchanged.
</commit_message>
<xml_diff>
--- a/results/Rede4genes_Expressao_Datasets.xlsx
+++ b/results/Rede4genes_Expressao_Datasets.xlsx
@@ -59,7 +59,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +76,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+        <bgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -105,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -132,6 +138,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -946,60 +955,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Gene</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>O que a literatura diz (não HPA)</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Nível confirmado no HPA (screenshot da usuária, 28/08/2026)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>O que a literatura diz</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Implicação para POP/SUI</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Link para conferir nível exato (HPA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Link para conferir (KREMEN1 ainda pendente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="220" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
           <t>CALML5</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>Proteína ligante de cálcio específica de queratinócitos em diferenciação terminal, expressa em epitélio escamoso estratificado (originalmente descrita na epiderme). Página do HPA cataloga expressão em útero, vagina, endométrio e colo do útero, mas o nível exato não veio no resumo de busca.</t>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>CONFIRMADO por imuno-histoquímica (anticorpo HPA040725) e RNA (GTEx): Vagina - proteína Low (células epiteliais escamosas), RNA 272,7 nTPM. Cérvice - proteína Medium (células epiteliais escamosas; glandulares = Not detected), RNA 198,9 nTPM. Overview de proteína: Skin/Breast/Salivary gland = High; Cervix/Tonsil = Medium; Vagina/Oral mucosa = Low; resto do corpo = Not detected.</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Vagina/colo/ectocérvice SÃO epitélio escamoso estratificado (mesma família tecidual da pele) — biologicamente plausível que CALML5 seja expressa aí de forma real, reforçando a hipótese de cornificação/diferenciação epitelial alterada já discutida.</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="inlineStr">
+          <t>Proteína ligante de cálcio de queratinócitos em diferenciação terminal, associada a TGM3 no envelope cornificado (já citado no rascunho da usuária).</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Expressão real, substancial e ESPECÍFICA de células epiteliais escamosas (não glandulares) em vagina e cérvice humanas — exatamente o tipo celular da hipótese de cornificação/diferenciação epitelial. Isso NÃO prova que CALML5 muda entre POP/SUI e controle (é expressão basal em tecido saudável do GTEx, não comparação de doença) — mas resolve a dúvida de fundo: CALML5 não é um gene obscuro/mal expresso nesse tipo de tecido, é um gene real e robustamente expresso lá. Isso enfraquece (não elimina) a preocupação de falso positivo técnico no rato: o padrão 0 nas 3 Untreated / valores altos em 2 das 3 Treated é mais compatível com indução biológica real (liga/desliga) do que com o gene simplesmente "não existir" nesse tecido. A limitação estatística de n=3 por grupo no rato continua de pé — isso é sobre poder amostral, não sobre se o gene é real.</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>https://www.proteinatlas.org/ENSG00000178372-CALML5/tissue</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>KREMEN1</t>
@@ -1007,15 +1027,20 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Receptor transmembrana que forma complexo com DKK1 e LRP5/LRP6, regulador central da via Wnt/beta-catenina (inibe endocitando os correceptores LRP5/6). HPA cataloga expressão em cérvice (ecto e endocérvice), tuba uterina, ovário, útero e vagina.</t>
+          <t>AINDA NÃO CONFERIDO — mesma checagem que você fez para CALML5, faça para KREMEN1 na mesma página (Tissue &gt; Vagina / Cervix / Uterus) e me manda print se quiser que eu documente aqui também.</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Via Wnt é conhecida por regular renovação/diferenciação epitelial e remodelação de tecido conjuntivo — plausível biologicamente que KREMEN1 alterado contribua tanto para a via epitelial (POP) quanto para reparo tecidual após lesão (SUI), mas isso é inferência de mecanismo geral, não medição direta no tecido pélvico.</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
+          <t>Receptor transmembrana que forma complexo com DKK1 e LRP5/LRP6, regulador central da via Wnt/beta-catenina (inibe endocitando os correceptores LRP5/6).</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Via Wnt regula renovação/diferenciação epitelial e remodelação de tecido conjuntivo — plausível para POP (passivo) e SUI (reparo pós-lesão), mas ainda é inferência de mecanismo geral até você confirmar o nível real no HPA.</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>https://www.proteinatlas.org/ENSG00000183762-KREMEN1/tissue</t>
         </is>
@@ -1024,7 +1049,9 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>